<commit_message>
audit(2026-05-25 PM): backfill PR #104 link in workbook
</commit_message>
<xml_diff>
--- a/audits/daily_usability_audit_2026-05-25.xlsx
+++ b/audits/daily_usability_audit_2026-05-25.xlsx
@@ -499,6 +499,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -649,6 +650,7 @@
         <v>9.5</v>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
@@ -665,6 +667,7 @@
         <v>9.76</v>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
@@ -677,6 +680,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
@@ -685,7 +689,7 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>chaos_tester #84  |  my_website #55  |  funder-finder (Toast aria-label, committed locally)</t>
+          <t>chaos_tester #84  |  my_website #55  |  funder-finder #104</t>
         </is>
       </c>
     </row>
@@ -9698,7 +9702,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Branch pushed; PR opening below in this run</t>
+          <t>https://github.com/SpikeyCoder/funder-finder/pull/104</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -9717,6 +9721,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>

</xml_diff>